<commit_message>
Add snapshot tenure and hiring cohorts including current staff
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EkCfTcQuoMNdgR3LAzHFSc
</commit_message>
<xml_diff>
--- a/srok_raboty_bronirovanie_kontrol.xlsx
+++ b/srok_raboty_bronirovanie_kontrol.xlsx
@@ -8,11 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="По должностям (ушли)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Медиана для графика" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Количество для графика" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отделы по годам" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действующие" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все записи" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез на дату" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Когорты найма" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Медиана для графика" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Количество для графика" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отделы по годам" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действующие" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все записи" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,6 +140,88 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Средний стаж работающих на дату, дни</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Срез на дату'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Срез на дату'!$A$2:$B$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Срез на дату'!$D$2:$D$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -282,7 +366,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -427,7 +511,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -576,12 +660,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="4320000"/>
+    <ext cx="7200000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -627,6 +711,33 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1482,124 +1593,295 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Должность</t>
-        </is>
-      </c>
-      <c r="B1" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C1" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D1" t="n">
-        <v>2026</v>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Дата среза</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Отдел</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Работало, чел</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Средний стаж, дн</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Медиана, дн</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Стаж &lt;90 дн, %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Стаж &gt;1 года, %</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Бронирование: Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>54</v>
+          <t>31.12.2024</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>505</v>
+        <v>14</v>
       </c>
       <c r="D2" t="n">
-        <v>46</v>
+        <v>381</v>
+      </c>
+      <c r="E2" t="n">
+        <v>378</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Бронирование: Руководитель/старший</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>67</v>
+          <t>31.12.2024</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>1582</v>
+        <v>19</v>
+      </c>
+      <c r="D3" t="n">
+        <v>209</v>
+      </c>
+      <c r="E3" t="n">
+        <v>176</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Бронирование: Специалист по бронированию</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>10</v>
+          <t>31.12.2024</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="D4" t="n">
-        <v>422</v>
+        <v>282</v>
+      </c>
+      <c r="E4" t="n">
+        <v>267</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Контроль: Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>111</v>
+          <t>31.12.2025</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>110</v>
+        <v>17</v>
       </c>
       <c r="D5" t="n">
-        <v>128</v>
+        <v>369</v>
+      </c>
+      <c r="E5" t="n">
+        <v>273</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.41</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Контроль: Менеджер 2/2</t>
-        </is>
+          <t>31.12.2025</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>23</v>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>268</v>
+      </c>
+      <c r="E6" t="n">
+        <v>177</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Контроль: Отдел контроля поездок</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>149</v>
+          <t>31.12.2025</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>504</v>
+        <v>40</v>
       </c>
       <c r="D7" t="n">
-        <v>848</v>
+        <v>311</v>
+      </c>
+      <c r="E7" t="n">
+        <v>209</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Контроль: Руководитель/старший</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>114</v>
+          <t>14.10.2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>27</v>
+      </c>
+      <c r="D8" t="n">
+        <v>287</v>
+      </c>
+      <c r="E8" t="n">
+        <v>125</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>14.10.2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>26</v>
+      </c>
+      <c r="D9" t="n">
+        <v>370</v>
+      </c>
+      <c r="E9" t="n">
+        <v>358</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>14.10.2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>53</v>
+      </c>
+      <c r="D10" t="n">
+        <v>328</v>
+      </c>
+      <c r="E10" t="n">
+        <v>212</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.38</v>
       </c>
     </row>
   </sheetData>
@@ -1609,6 +1891,258 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Год найма</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Отдел</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Принято</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ещё работают</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>% остались</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Средний срок работы всех (до ухода или до сегодня), дн</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F3" t="n">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>48</v>
+      </c>
+      <c r="D4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F4" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>21</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F5" t="n">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>29</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F6" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="n">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F7" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>28</v>
+      </c>
+      <c r="D8" t="n">
+        <v>19</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F8" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>17</v>
+      </c>
+      <c r="D9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F9" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>45</v>
+      </c>
+      <c r="D10" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F10" t="n">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1644,13 +2178,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>505</v>
       </c>
       <c r="D2" t="n">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -1660,13 +2194,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="4">
@@ -1676,13 +2207,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>422</v>
       </c>
     </row>
     <row r="5">
@@ -1692,13 +2223,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>111</v>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6">
@@ -1707,14 +2238,8 @@
           <t>Контроль: Менеджер 2/2</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -1724,13 +2249,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>149</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>504</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>848</v>
       </c>
     </row>
     <row r="8">
@@ -1740,13 +2265,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1755,7 +2274,154 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Должность</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Бронирование: Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Бронирование: Руководитель/старший</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Бронирование: Специалист по бронированию</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Контроль: Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Контроль: Менеджер 2/2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Контроль: Отдел контроля поездок</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Контроль: Руководитель/старший</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1822,7 +2488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2182,7 +2848,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add breakdown by department, hire year, status and time-to-leave buckets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EkCfTcQuoMNdgR3LAzHFSc
</commit_message>
<xml_diff>
--- a/srok_raboty_bronirovanie_kontrol.xlsx
+++ b/srok_raboty_bronirovanie_kontrol.xlsx
@@ -7,14 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="По должностям (ушли)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез на дату" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Когорты найма" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Медиана для графика" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Количество для графика" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отделы по годам" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действующие" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все записи" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Разбивка (менеджеры)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="По должностям (ушли)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез на дату" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Когорты найма" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Медиана для графика" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Количество для графика" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отделы по годам" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действующие" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все записи" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1053,11 +1054,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1068,37 +1079,57 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Должность</t>
+          <t>Год найма</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Год ухода</t>
+          <t>Принято</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ушло</t>
+          <t>Работают</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Средний срок, дн</t>
+          <t>% работают</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Медиана, дн</t>
+          <t>Ушли</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Ушли &lt;90 дн</t>
+          <t>до 3 дней</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>% &lt;90 дн</t>
+          <t>4–7 дней</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>8–30 дней</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>31–60 дней</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>61–180 дней</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>больше 6 мес.</t>
         </is>
       </c>
     </row>
@@ -1108,28 +1139,38 @@
           <t>Бронирование</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
+      <c r="B2" t="n">
+        <v>2024</v>
       </c>
       <c r="C2" t="n">
-        <v>2024</v>
+        <v>14</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E2" t="n">
-        <v>63</v>
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.14</v>
       </c>
       <c r="F2" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -1138,28 +1179,38 @@
           <t>Бронирование</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
+      <c r="B3" t="n">
+        <v>2025</v>
       </c>
       <c r="C3" t="n">
-        <v>2025</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
-      <c r="E3" t="n">
-        <v>269</v>
+      <c r="E3" s="2" t="n">
+        <v>0.6</v>
       </c>
       <c r="F3" t="n">
-        <v>360</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>0.33</v>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1168,28 +1219,38 @@
           <t>Бронирование</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
+      <c r="B4" t="n">
+        <v>2026</v>
       </c>
       <c r="C4" t="n">
-        <v>2026</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" t="n">
-        <v>77</v>
+        <v>19</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.68</v>
       </c>
       <c r="F4" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="G4" t="n">
-        <v>7</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1198,28 +1259,38 @@
           <t>Контроль</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
+      <c r="B5" t="n">
+        <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>2024</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" t="n">
-        <v>54</v>
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.19</v>
       </c>
       <c r="F5" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>0.83</v>
+      <c r="L5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -1228,28 +1299,38 @@
           <t>Контроль</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
+      <c r="B6" t="n">
+        <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>2025</v>
+        <v>29</v>
       </c>
       <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F6" t="n">
         <v>20</v>
       </c>
-      <c r="E6" t="n">
-        <v>137</v>
-      </c>
-      <c r="F6" t="n">
-        <v>110</v>
-      </c>
       <c r="G6" t="n">
-        <v>7</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>0.35</v>
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" t="n">
+        <v>9</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1258,58 +1339,583 @@
           <t>Контроль</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
+      <c r="B7" t="n">
+        <v>2026</v>
       </c>
       <c r="C7" t="n">
-        <v>2026</v>
+        <v>17</v>
       </c>
       <c r="D7" t="n">
         <v>11</v>
       </c>
-      <c r="E7" t="n">
-        <v>130</v>
+      <c r="E7" s="2" t="n">
+        <v>0.65</v>
       </c>
       <c r="F7" t="n">
-        <v>128</v>
+        <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0.36</v>
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Контроль</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Менеджер 2/2</t>
-        </is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2024</v>
       </c>
       <c r="C8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="F8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" t="n">
+        <v>9</v>
+      </c>
+      <c r="L8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C9" t="n">
+        <v>34</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F9" t="n">
+        <v>22</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>9</v>
+      </c>
+      <c r="L9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>2026</v>
       </c>
-      <c r="D8" t="n">
+      <c r="C10" t="n">
+        <v>45</v>
+      </c>
+      <c r="D10" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
         <v>2</v>
       </c>
-      <c r="E8" t="n">
-        <v>12</v>
-      </c>
-      <c r="F8" t="n">
-        <v>12</v>
-      </c>
-      <c r="G8" t="n">
+      <c r="I10" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Самый успешный найм (по числу оставшихся)</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="n"/>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="1" t="n"/>
+      <c r="J12" s="1" t="n"/>
+      <c r="K12" s="1" t="n"/>
+      <c r="L12" s="1" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>по числу: 2026 (19 из 28)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>по доле: 2026 (68%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>по числу: 2026 (11 из 17)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>по доле: 2026 (65%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>по числу: 2026 (30 из 45)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>по доле: 2026 (67%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Отдел</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Год ухода</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Ушло</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>до 3 дней</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>4–7 дней</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>8–30 дней</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="inlineStr">
+        <is>
+          <t>31–60 дней</t>
+        </is>
+      </c>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>61–180 дней</t>
+        </is>
+      </c>
+      <c r="L17" s="1" t="inlineStr">
+        <is>
+          <t>больше 6 мес.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="K18" t="n">
+        <v>4</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
         <v>1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>2</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>2</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C22" t="n">
+        <v>20</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>9</v>
+      </c>
+      <c r="L22" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C23" t="n">
+        <v>13</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C24" t="n">
+        <v>16</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="n">
+        <v>6</v>
+      </c>
+      <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>6</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C25" t="n">
+        <v>23</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>5</v>
+      </c>
+      <c r="K25" t="n">
+        <v>9</v>
+      </c>
+      <c r="L25" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Оба отдела</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C26" t="n">
+        <v>23</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>7</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>6</v>
+      </c>
+      <c r="L26" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1323,8 +1929,278 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Отдел</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Должность</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Год ухода</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ушло</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Средний срок, дн</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Медиана, дн</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Ушли &lt;90 дн</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>% &lt;90 дн</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>63</v>
+      </c>
+      <c r="F2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>269</v>
+      </c>
+      <c r="F3" t="n">
+        <v>360</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>77</v>
+      </c>
+      <c r="F4" t="n">
+        <v>35</v>
+      </c>
+      <c r="G4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>54</v>
+      </c>
+      <c r="F5" t="n">
+        <v>38</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137</v>
+      </c>
+      <c r="F6" t="n">
+        <v>110</v>
+      </c>
+      <c r="G6" t="n">
+        <v>7</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11</v>
+      </c>
+      <c r="E7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F7" t="n">
+        <v>128</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Менеджер 2/2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -1620,14 +2496,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -1872,14 +2748,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -1941,89 +2817,6 @@
       </c>
       <c r="D4" t="n">
         <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Должность</t>
-        </is>
-      </c>
-      <c r="B1" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C1" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D1" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Бронирование: Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Контроль: Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D3" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Контроль: Менеджер 2/2</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2038,8 +2831,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -2048,7 +2841,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Отдел</t>
+          <t>Должность</t>
         </is>
       </c>
       <c r="B1" t="n">
@@ -2064,33 +2857,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Бронирование (медиана, дн)</t>
+          <t>Бронирование: Менеджер (основной)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>360</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Контроль (медиана, дн)</t>
+          <t>Контроль: Менеджер (основной)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>110</v>
+        <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>94</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Контроль: Менеджер 2/2</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2105,8 +2914,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -2118,239 +2927,51 @@
           <t>Отдел</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Должность</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Год найма</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Человек</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Средний срок, дн</t>
-        </is>
+      <c r="B1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Бронирование</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Вечерний менеджер</t>
-        </is>
+          <t>Бронирование (медиана, дн)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>44</v>
       </c>
       <c r="C2" t="n">
-        <v>2026</v>
+        <v>360</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
-      </c>
-      <c r="E2" t="n">
-        <v>63</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Бронирование</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
+          <t>Контроль (медиана, дн)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>2024</v>
+        <v>110</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="n">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Бронирование</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Бронирование</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="n">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Бронирование</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Менеджер 2/2</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E6" t="n">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Контроль</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Вечерний менеджер</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Контроль</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" t="n">
-        <v>763</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Контроль</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D9" t="n">
-        <v>9</v>
-      </c>
-      <c r="E9" t="n">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Контроль</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Менеджер (основной)</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="n">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Контроль</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Менеджер 2/2</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D11" t="n">
-        <v>8</v>
-      </c>
-      <c r="E11" t="n">
-        <v>31</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2360,8 +2981,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -2370,6 +2991,261 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Отдел</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Должность</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Год найма</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Человек</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Средний срок, дн</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Вечерний менеджер</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Бронирование</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Менеджер 2/2</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Вечерний менеджер</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D9" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Менеджер (основной)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Контроль</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Менеджер 2/2</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" t="n">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H110"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>ФИО</t>
         </is>
       </c>

</xml_diff>